<commit_message>
Adding extension and mcp and other apps
</commit_message>
<xml_diff>
--- a/KG/sample_data/class_level_data_1.xlsx
+++ b/KG/sample_data/class_level_data_1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Iris\practice\GenAI\code\Batch_KG\sample_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63E77151-BCF9-4C3C-841C-AD39C7469863}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B96BB433-8EDD-4775-889F-F2BF26614EC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="736" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="736" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="JobGroups" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="926" uniqueCount="401">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="930" uniqueCount="401">
   <si>
     <t>id</t>
   </si>
@@ -1650,14 +1650,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="20.453125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="24.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1673,8 +1673,11 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F1" s="2" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1691,7 +1694,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>327</v>
       </c>
@@ -1707,8 +1710,11 @@
       <c r="E3" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>346</v>
       </c>
@@ -1724,8 +1730,11 @@
       <c r="E4" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F4" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>321</v>
       </c>
@@ -1741,8 +1750,11 @@
       <c r="E5" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F5" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>384</v>
       </c>

</xml_diff>